<commit_message>
Brass MTA in Heavy and Light; sizes can carry a make
A size heading can now end with a make, e.g. '3/4x1/2 Heavy'. The app shows
it as its own size button (make on a second line) and prints it on the bill.
Ashirvad brass MTA 3/4 x 1/2 is now Heavy 283 and Light 210 in the built-in
rates. Items with more than six sizes lay out four across where the phone is
wide enough, so the keypad and Add button stay on screen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H9ATNSb1ytNQiSAWXE3aDp
</commit_message>
<xml_diff>
--- a/deliver/Mangal-rates.xlsx
+++ b/deliver/Mangal-rates.xlsx
@@ -261,11 +261,6 @@
     <comment ref="K22" authorId="0" shapeId="0">
       <text>
         <t>The Tee row on your sheet is overwritten and crossed out. Please type the correct rate.</t>
-      </text>
-    </comment>
-    <comment ref="J23" authorId="0" shapeId="0">
-      <text>
-        <t>Your sheet has two rates here: H 283 and L 210. Which one should the app use? (If both are sold, tell me and I will add them as two items.)</t>
       </text>
     </comment>
     <comment ref="D25" authorId="0" shapeId="0">
@@ -636,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -646,10 +641,12 @@
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -766,6 +763,16 @@
       <c r="K6" s="4" t="inlineStr">
         <is>
           <t>1x1/2</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>3/4x1/2 Heavy</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>3/4x1/2 Light</t>
         </is>
       </c>
     </row>
@@ -799,6 +806,8 @@
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -836,6 +845,8 @@
       </c>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -873,6 +884,8 @@
       </c>
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -910,6 +923,8 @@
       </c>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
+      <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -941,6 +956,8 @@
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -972,6 +989,8 @@
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7" t="n"/>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1003,6 +1022,8 @@
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1038,6 +1059,8 @@
       <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="n"/>
       <c r="K14" s="7" t="n"/>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1069,6 +1092,8 @@
       <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
+      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1100,6 +1125,8 @@
       <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1131,6 +1158,8 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
+      <c r="L17" s="7" t="n"/>
+      <c r="M17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1162,6 +1191,8 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1193,6 +1224,8 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
       <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1224,6 +1257,8 @@
       </c>
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1263,6 +1298,8 @@
       <c r="K21" s="7" t="n">
         <v>214</v>
       </c>
+      <c r="L21" s="7" t="n"/>
+      <c r="M21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1312,6 +1349,8 @@
           <t>?</t>
         </is>
       </c>
+      <c r="L22" s="7" t="n"/>
+      <c r="M22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1343,13 +1382,15 @@
       </c>
       <c r="H23" s="7" t="n"/>
       <c r="I23" s="7" t="n"/>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
+      <c r="J23" s="7" t="n"/>
       <c r="K23" s="7" t="n">
         <v>413</v>
+      </c>
+      <c r="L23" s="7" t="n">
+        <v>283</v>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>210</v>
       </c>
     </row>
     <row r="24">
@@ -1388,6 +1429,8 @@
       <c r="K24" s="7" t="n">
         <v>192</v>
       </c>
+      <c r="L24" s="7" t="n"/>
+      <c r="M24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1421,6 +1464,8 @@
       <c r="I25" s="7" t="n"/>
       <c r="J25" s="7" t="n"/>
       <c r="K25" s="7" t="n"/>
+      <c r="L25" s="7" t="n"/>
+      <c r="M25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1460,6 +1505,8 @@
       </c>
       <c r="J26" s="7" t="n"/>
       <c r="K26" s="7" t="n"/>
+      <c r="L26" s="7" t="n"/>
+      <c r="M26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1497,6 +1544,8 @@
       </c>
       <c r="J27" s="7" t="n"/>
       <c r="K27" s="7" t="n"/>
+      <c r="L27" s="7" t="n"/>
+      <c r="M27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1536,6 +1585,8 @@
       </c>
       <c r="J28" s="7" t="n"/>
       <c r="K28" s="7" t="n"/>
+      <c r="L28" s="7" t="n"/>
+      <c r="M28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1569,6 +1620,8 @@
       <c r="I29" s="7" t="n"/>
       <c r="J29" s="7" t="n"/>
       <c r="K29" s="7" t="n"/>
+      <c r="L29" s="7" t="n"/>
+      <c r="M29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1600,6 +1653,8 @@
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="7" t="n"/>
       <c r="K30" s="7" t="n"/>
+      <c r="L30" s="7" t="n"/>
+      <c r="M30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1633,6 +1688,8 @@
       <c r="I31" s="7" t="n"/>
       <c r="J31" s="7" t="n"/>
       <c r="K31" s="7" t="n"/>
+      <c r="L31" s="7" t="n"/>
+      <c r="M31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1666,6 +1723,8 @@
       <c r="I32" s="7" t="n"/>
       <c r="J32" s="7" t="n"/>
       <c r="K32" s="7" t="n"/>
+      <c r="L32" s="7" t="n"/>
+      <c r="M32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1697,6 +1756,8 @@
       <c r="I33" s="7" t="n"/>
       <c r="J33" s="7" t="n"/>
       <c r="K33" s="7" t="n"/>
+      <c r="L33" s="7" t="n"/>
+      <c r="M33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1728,6 +1789,8 @@
       <c r="I34" s="7" t="n"/>
       <c r="J34" s="7" t="n"/>
       <c r="K34" s="7" t="n"/>
+      <c r="L34" s="7" t="n"/>
+      <c r="M34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -1765,6 +1828,8 @@
       <c r="I35" s="7" t="n"/>
       <c r="J35" s="7" t="n"/>
       <c r="K35" s="7" t="n"/>
+      <c r="L35" s="7" t="n"/>
+      <c r="M35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1796,6 +1861,8 @@
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="7" t="n"/>
       <c r="K36" s="7" t="n"/>
+      <c r="L36" s="7" t="n"/>
+      <c r="M36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -1827,6 +1894,8 @@
       <c r="I37" s="7" t="n"/>
       <c r="J37" s="7" t="n"/>
       <c r="K37" s="7" t="n"/>
+      <c r="L37" s="7" t="n"/>
+      <c r="M37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -1858,6 +1927,8 @@
       </c>
       <c r="J38" s="7" t="n"/>
       <c r="K38" s="7" t="n"/>
+      <c r="L38" s="7" t="n"/>
+      <c r="M38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -1897,6 +1968,8 @@
       <c r="K39" s="7" t="n">
         <v>139.4</v>
       </c>
+      <c r="L39" s="7" t="n"/>
+      <c r="M39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -1934,6 +2007,8 @@
       <c r="K40" s="7" t="n">
         <v>152.1</v>
       </c>
+      <c r="L40" s="7" t="n"/>
+      <c r="M40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -1973,6 +2048,8 @@
       <c r="K41" s="7" t="n">
         <v>254.8</v>
       </c>
+      <c r="L41" s="7" t="n"/>
+      <c r="M41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -2012,6 +2089,8 @@
           <t>?</t>
         </is>
       </c>
+      <c r="L42" s="7" t="n"/>
+      <c r="M42" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2025,7 +2104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2127,84 +2206,91 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
+          <t>Same size in two makes (heavy and light): give each its own column, with the make after the size, for example 3/4x1/2 Heavy and 3/4x1/2 Light. The app shows them as two size buttons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
           <t>New brand: just use the new brand name in column A. It appears in the app as a new brand button.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Rules the app checks</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>Keep the heading row starting with Brand, Type, Item. Rates are numbers only (62 or 21.30). The same item and size must not appear twice.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Type decides the discount group: all Plain items of a brand share one discount, all Brass items another, Pipe another.</t>
+          <t>Keep the heading row starting with Brand, Type, Item. Rates are numbers only (62 or 21.30). The same item and size must not appear twice.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Items of type Brass are printed on the bill as "Tee (Brass)". Plain and Pipe items are printed without brackets.</t>
+          <t>Type decides the discount group: all Plain items of a brand share one discount, all Brass items another, Pipe another.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
+          <t>Items of type Brass are printed on the bill as "Tee (Brass)". Plain and Pipe items are printed without brackets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
           <t>If the sheet has a mistake, the app keeps using the last good rates and shows which row and column is wrong (tap "Rates updated" in the app).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>To connect this sheet to the app (one time)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>1. Upload this file to Google Drive and open it with Google Sheets.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>2. File &gt; Share &gt; Publish to web. Choose the "Rates" tab and "Comma-separated values (.csv)". Press Publish.</t>
+          <t>1. Upload this file to Google Drive and open it with Google Sheets.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
+          <t>2. File &gt; Share &gt; Publish to web. Choose the "Rates" tab and "Comma-separated values (.csv)". Press Publish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
           <t>3. Copy the link it gives and send it to me. I will put it in the app. After that, every phone picks up your changes when it has internet (Google can take about 5 minutes).</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>Source of the rates: your two rate-sheet photos dated 6 Oct 2026 (Ashirvad and Supreme). They are not confirmed yet.</t>
         </is>
@@ -2221,7 +2307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2504,27 +2590,27 @@
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>Ashirvad</t>
+          <t>Supreme</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Brass</t>
+          <t>Pipe</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>Pipe SDR 11</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>3/4x1/2</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Your sheet has two rates here: H 283 and L 210. Which one should the app use? (If both are sold, tell me and I will add them as two items.)</t>
+          <t>It looks like 219.33, which seems low next to 658 for 1". Please type the correct rate.</t>
         </is>
       </c>
     </row>
@@ -2536,22 +2622,22 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Pipe</t>
+          <t>Plain</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Pipe SDR 11</t>
+          <t>Elbow</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>1 1/4x1</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>It looks like 219.33, which seems low next to 658 for 1". Please type the correct rate.</t>
+          <t>Empty on your sheet. Type the rate, or empty this box if you do not sell this size.</t>
         </is>
       </c>
     </row>
@@ -2568,17 +2654,17 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Elbow</t>
+          <t>Socket</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>1 1/4x1</t>
+          <t>1x3/4</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Empty on your sheet. Type the rate, or empty this box if you do not sell this size.</t>
+          <t>Overwritten on your sheet. It looks like 36.90. Please type the correct rate.</t>
         </is>
       </c>
     </row>
@@ -2595,17 +2681,17 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>Socket</t>
+          <t>Union</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>1x3/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Overwritten on your sheet. It looks like 36.90. Please type the correct rate.</t>
+          <t>Empty on your sheet. Type the rate, or empty this box if you do not sell this size.</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2708,7 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Ball Valve</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -2632,7 +2718,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Empty on your sheet. Type the rate, or empty this box if you do not sell this size.</t>
+          <t>Smudged on your sheet. It looks like 220.10. Please type the correct rate.</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2735,17 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Ball Valve</t>
+          <t>Over Step Bend</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>1 1/4</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Smudged on your sheet. It looks like 220.10. Please type the correct rate.</t>
+          <t>Empty on your sheet. Type the rate, or empty this box if you do not sell this size. There is also a side note "3/4: 81.20, 1: 199.20" next to this row. Which item is that for?</t>
         </is>
       </c>
     </row>
@@ -2676,17 +2762,17 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Over Step Bend</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>1 1/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Empty on your sheet. Type the rate, or empty this box if you do not sell this size. There is also a side note "3/4: 81.20, 1: 199.20" next to this row. Which item is that for?</t>
+          <t>Your MTA row is marked "PVC" with sizes 3/4x1/2 = 31.50, 1x3/4 = 33.60, 1 1/4x1 = 68. What are the plain MTA rates for 3/4, 1 and 1 1/4?</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2794,7 @@
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
@@ -2735,7 +2821,7 @@
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1 1/4</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
@@ -2757,17 +2843,17 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>C Bend</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>1 1/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Your MTA row is marked "PVC" with sizes 3/4x1/2 = 31.50, 1x3/4 = 33.60, 1 1/4x1 = 68. What are the plain MTA rates for 3/4, 1 and 1 1/4?</t>
+          <t>These numbers are written next to "C Bend" under the Elbow row on your sheet. Please confirm they are the C Bend rates.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2875,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -2816,7 +2902,7 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1 1/4</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
@@ -2833,12 +2919,12 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Plain</t>
+          <t>Brass</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>C Bend</t>
+          <t>Elbow</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
@@ -2848,7 +2934,7 @@
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>These numbers are written next to "C Bend" under the Elbow row on your sheet. Please confirm they are the C Bend rates.</t>
+          <t>It looks like 483.60 or 482.60. Please type the correct rate.</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2951,7 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Elbow</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
@@ -2875,7 +2961,7 @@
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>It looks like 483.60 or 482.60. Please type the correct rate.</t>
+          <t>Overwritten on your sheet. It looks like 724.40. Please type the correct rate.</t>
         </is>
       </c>
     </row>
@@ -2892,61 +2978,34 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>FTA</t>
         </is>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>1 1/4</t>
+          <t>1x1/2</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Overwritten on your sheet. It looks like 724.40. Please type the correct rate.</t>
+          <t>Overwritten on your sheet. It looks like 116.10. Please type the correct rate.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>Supreme</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>Brass</t>
-        </is>
-      </c>
+          <t>Ashirvad</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr"/>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>FTA</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>1x1/2</t>
-        </is>
-      </c>
+          <t>Reducing MTA</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr"/>
       <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>Overwritten on your sheet. It looks like 116.10. Please type the correct rate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>Ashirvad</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="inlineStr"/>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>Reducing MTA</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr"/>
-      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>Your sheet has a hand-written note "Reducing MTA 54 ... 64" above the brass table. Which sizes are these, and should it be an item in the app?</t>
         </is>

</xml_diff>